<commit_message>
Aura: mano de obra por m² (USD 340) y sin duplicar instalaciones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PL4fade9uMUQLM1tmUvUUs
</commit_message>
<xml_diff>
--- a/URBANSIP/AURA/Aura_Esencial_Presupuesto_v1.xlsx
+++ b/URBANSIP/AURA/Aura_Esencial_Presupuesto_v1.xlsx
@@ -117,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -161,6 +161,7 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1427,7 +1428,7 @@
         </is>
       </c>
       <c r="C32" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="16" t="n">
         <v>850000</v>
@@ -1440,14 +1441,14 @@
         <f>E32/$B$2</f>
         <v/>
       </c>
-      <c r="G32" s="18" t="inlineStr">
-        <is>
-          <t>DUDA</t>
+      <c r="G32" s="20" t="inlineStr">
+        <is>
+          <t>CORREGIDO</t>
         </is>
       </c>
       <c r="H32" s="19" t="inlineStr">
         <is>
-          <t>La planilla de mano de obra también tiene días de instalaciones (13 días). Puede estar contada dos veces.</t>
+          <t>Se elimina: la mano de obra por m² de obra gris ya incluye instalaciones (Excel de costos: 'OBRA GRIS CON INST + DURLOCK').</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1586,7 @@
         </is>
       </c>
       <c r="C37" s="14" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="D37" s="16" t="n">
         <v>60000</v>
@@ -1598,14 +1599,14 @@
         <f>E37/$B$2</f>
         <v/>
       </c>
-      <c r="G37" s="18" t="inlineStr">
-        <is>
-          <t>DUDA</t>
+      <c r="G37" s="20" t="inlineStr">
+        <is>
+          <t>CORREGIDO</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>Ídem mano de obra sanitaria.</t>
+          <t>Se elimina: la mano de obra por m² de obra gris ya incluye instalaciones (Excel de costos: 'OBRA GRIS CON INST + DURLOCK').</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2315,7 @@
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>MANO DE OBRA (cuadrilla propia, planilla 'Mano de obra Aura')</t>
+          <t>MANO DE OBRA (por m², según Excel de costos: costo USD 340/m²)</t>
         </is>
       </c>
       <c r="B63" s="10" t="n"/>
@@ -2328,19 +2329,21 @@
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>Montaje del kit SIP (22 días × $240.000)</t>
+          <t>Mano de obra obra gris: montaje kit + instalaciones + durlock (u$s/m²)</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>gl</t>
-        </is>
-      </c>
-      <c r="C64" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="16" t="n">
-        <v>5280000</v>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C64" s="14">
+        <f>$D$2</f>
+        <v/>
+      </c>
+      <c r="D64" s="31">
+        <f>204*$B$2</f>
+        <v/>
       </c>
       <c r="E64" s="16">
         <f>C64*D64</f>
@@ -2357,26 +2360,28 @@
       </c>
       <c r="H64" s="19" t="inlineStr">
         <is>
-          <t>Cuadrilla de 3: oficial especializado + oficial + ayudante.</t>
+          <t>USD 204/m² (de los cuales USD 108,8 son el montaje del kit).</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
         <is>
-          <t>Obra gris y terminaciones (54 días × $280.000)</t>
+          <t>Mano de obra terminaciones (u$s/m²)</t>
         </is>
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>gl</t>
-        </is>
-      </c>
-      <c r="C65" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="16" t="n">
-        <v>15120000</v>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C65" s="14">
+        <f>$D$2</f>
+        <v/>
+      </c>
+      <c r="D65" s="31">
+        <f>136*$B$2</f>
+        <v/>
       </c>
       <c r="E65" s="16">
         <f>C65*D65</f>
@@ -2386,14 +2391,14 @@
         <f>E65/$B$2</f>
         <v/>
       </c>
-      <c r="G65" s="18" t="inlineStr">
-        <is>
-          <t>DUDA</t>
+      <c r="G65" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H65" s="19" t="inlineStr">
         <is>
-          <t>Incluye 13 días de instalaciones (ver mano de obra sanitaria y eléctrica). ¿Por qué $280.000 y no $240.000 por día?</t>
+          <t>USD 136/m².</t>
         </is>
       </c>
     </row>
@@ -2756,22 +2761,22 @@
       </c>
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>DEFINIDO</t>
         </is>
       </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
-          <t>Mano de obra (planilla MdeO)</t>
+          <t>Mano de obra</t>
         </is>
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>El 'u$s/m² llave en mano' (263,83) toma los 54 días sin kit, los escala a 76 días (agrega los 22 días del kit a precio de obra gris) y además suma el kit (60 u$s/m²): el montaje del kit queda contado dos veces. También usa dólar $1.450 y $1.330. Costo real: $5.280.000 + $15.120.000 = $20.400.000 ≈ USD 13.160 (USD 180/m²). Ya corregido en este presupuesto.</t>
+          <t>Adrián: la mano de obra se cobra por m². Costo USD 340/m² (obra gris con instalaciones y durlock 204 + terminaciones 136), venta 1,5 × = USD 510/m². La planilla 'Mano de obra Aura' (por jornales) queda solo como control: da USD 180/m² y además cuenta dos veces el montaje del kit.</t>
         </is>
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>−6.100 de costo</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2886,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>DUDA</t>
+          <t>DEFINIDO</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
@@ -2891,12 +2896,12 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Tu Excel de costos usa 340 u$s/m² de mano de obra como base del margen (venta 510). El costo real da 180. Con 1,5 × 180 la ganancia baja a ≈ USD 6.580. ¿Sobre qué mano de obra se aplica el 1,5?</t>
+          <t>Margen = 1,5 × mano de obra por m² (USD 340). Ganancia ≈ USD 12.410.</t>
         </is>
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>Decisión tuya</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2906,7 +2911,7 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>DUDA</t>
+          <t>CORREGIDO</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
@@ -2916,12 +2921,12 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Mano de obra sanitaria y eléctrica en materiales ($4.090.000) + 13 días en la planilla de mano de obra.</t>
+          <t>Mano de obra sanitaria y eléctrica de la hoja Materiales ($4.090.000) eliminada: ya está en la mano de obra por m² de obra gris ('con instalaciones').</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>hasta −2.640</t>
+          <t>−2.640</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3046,7 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Kit a $240.000/día, resto a $280.000/día.</t>
+          <t>Kit a $240.000/día, resto a $280.000/día (solo afecta la planilla de control por jornales).</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">

</xml_diff>